<commit_message>
cambios en el login
</commit_message>
<xml_diff>
--- a/docs/Plan_de_mejora_app_circuitos_smd.xlsx
+++ b/docs/Plan_de_mejora_app_circuitos_smd.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
@@ -575,6 +575,10 @@
 </styleSheet>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>

</xml_diff>